<commit_message>
claude api integrated and tested
</commit_message>
<xml_diff>
--- a/kyc_process_results.xlsx
+++ b/kyc_process_results.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L748"/>
+  <dimension ref="A1:L758"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43939,6 +43939,550 @@
         </is>
       </c>
     </row>
+    <row r="749">
+      <c r="A749" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B749" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000050</t>
+        </is>
+      </c>
+      <c r="C749" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D749" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E749" s="4" t="inlineStr">
+        <is>
+          <t>Mohanish Kumar Sinha</t>
+        </is>
+      </c>
+      <c r="F749" s="4" t="inlineStr">
+        <is>
+          <t>RALAS AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="G749" s="4" t="inlineStr">
+        <is>
+          <t>DHAMTARI</t>
+        </is>
+      </c>
+      <c r="H749" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I749" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J749" s="4" t="inlineStr"/>
+      <c r="K749" s="3" t="inlineStr"/>
+      <c r="L749" s="4" t="inlineStr">
+        <is>
+          <t>T2D86537</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B750" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000049</t>
+        </is>
+      </c>
+      <c r="C750" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D750" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E750" s="4" t="inlineStr">
+        <is>
+          <t>DINESH SONI</t>
+        </is>
+      </c>
+      <c r="F750" s="4" t="inlineStr">
+        <is>
+          <t>RALAS AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="G750" s="4" t="inlineStr">
+        <is>
+          <t>DHAMTARI</t>
+        </is>
+      </c>
+      <c r="H750" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I750" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J750" s="4" t="inlineStr"/>
+      <c r="K750" s="3" t="inlineStr"/>
+      <c r="L750" s="4" t="inlineStr">
+        <is>
+          <t>T6E56018</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B751" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000048</t>
+        </is>
+      </c>
+      <c r="C751" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D751" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E751" s="4" t="inlineStr">
+        <is>
+          <t>TILAK CHAND DEWANGAN</t>
+        </is>
+      </c>
+      <c r="F751" s="4" t="inlineStr">
+        <is>
+          <t>RALAS AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="G751" s="4" t="inlineStr">
+        <is>
+          <t>DHAMTARI</t>
+        </is>
+      </c>
+      <c r="H751" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I751" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J751" s="4" t="inlineStr">
+        <is>
+          <t>COD Document Validation Failed: COD Vehicle Model 'TATA ECE' does not match expected old vehicle model 'Ace'</t>
+        </is>
+      </c>
+      <c r="K751" s="3" t="inlineStr"/>
+      <c r="L751" s="4" t="inlineStr">
+        <is>
+          <t>T1E91511</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B752" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000017</t>
+        </is>
+      </c>
+      <c r="C752" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D752" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E752" s="4" t="inlineStr">
+        <is>
+          <t>Mayank .</t>
+        </is>
+      </c>
+      <c r="F752" s="4" t="inlineStr">
+        <is>
+          <t>B R BALAJI LLP</t>
+        </is>
+      </c>
+      <c r="G752" s="4" t="inlineStr">
+        <is>
+          <t>JAGDALPUR</t>
+        </is>
+      </c>
+      <c r="H752" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I752" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J752" s="4" t="inlineStr">
+        <is>
+          <t>COD Document Validation Failed: COD Vehicle Model 'ZEN MPI LX' does not match expected old vehicle model 'Zen lx'
+Missing Disclaimer Document</t>
+        </is>
+      </c>
+      <c r="K752" s="3" t="inlineStr"/>
+      <c r="L752" s="4" t="inlineStr">
+        <is>
+          <t>T2D85723</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B753" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000161</t>
+        </is>
+      </c>
+      <c r="C753" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D753" s="4" t="inlineStr">
+        <is>
+          <t>AD Bhubaneshwar</t>
+        </is>
+      </c>
+      <c r="E753" s="4" t="inlineStr">
+        <is>
+          <t>ANAND TULSIAN</t>
+        </is>
+      </c>
+      <c r="F753" s="4" t="inlineStr">
+        <is>
+          <t>G N AUTONATION LLP</t>
+        </is>
+      </c>
+      <c r="G753" s="4" t="inlineStr">
+        <is>
+          <t>NEW_SAMBALPUR</t>
+        </is>
+      </c>
+      <c r="H753" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I753" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J753" s="4" t="inlineStr">
+        <is>
+          <t>Missing Ledger Document</t>
+        </is>
+      </c>
+      <c r="K753" s="3" t="inlineStr"/>
+      <c r="L753" s="4" t="inlineStr">
+        <is>
+          <t>T1D88570</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B754" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000048</t>
+        </is>
+      </c>
+      <c r="C754" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D754" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E754" s="4" t="inlineStr">
+        <is>
+          <t>TILAK CHAND DEWANGAN</t>
+        </is>
+      </c>
+      <c r="F754" s="4" t="inlineStr">
+        <is>
+          <t>RALAS AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="G754" s="4" t="inlineStr">
+        <is>
+          <t>DHAMTARI</t>
+        </is>
+      </c>
+      <c r="H754" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I754" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J754" s="4" t="inlineStr"/>
+      <c r="K754" s="3" t="inlineStr"/>
+      <c r="L754" s="4" t="inlineStr">
+        <is>
+          <t>T1E91511</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B755" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000017</t>
+        </is>
+      </c>
+      <c r="C755" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D755" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E755" s="4" t="inlineStr">
+        <is>
+          <t>Mayank .</t>
+        </is>
+      </c>
+      <c r="F755" s="4" t="inlineStr">
+        <is>
+          <t>B R BALAJI LLP</t>
+        </is>
+      </c>
+      <c r="G755" s="4" t="inlineStr">
+        <is>
+          <t>JAGDALPUR</t>
+        </is>
+      </c>
+      <c r="H755" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I755" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J755" s="4" t="inlineStr">
+        <is>
+          <t>Missing Disclaimer Document</t>
+        </is>
+      </c>
+      <c r="K755" s="3" t="inlineStr"/>
+      <c r="L755" s="4" t="inlineStr">
+        <is>
+          <t>T2D85723</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B756" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000161</t>
+        </is>
+      </c>
+      <c r="C756" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D756" s="4" t="inlineStr">
+        <is>
+          <t>AD Bhubaneshwar</t>
+        </is>
+      </c>
+      <c r="E756" s="4" t="inlineStr">
+        <is>
+          <t>ANAND TULSIAN</t>
+        </is>
+      </c>
+      <c r="F756" s="4" t="inlineStr">
+        <is>
+          <t>G N AUTONATION LLP</t>
+        </is>
+      </c>
+      <c r="G756" s="4" t="inlineStr">
+        <is>
+          <t>NEW_SAMBALPUR</t>
+        </is>
+      </c>
+      <c r="H756" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I756" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J756" s="4" t="inlineStr"/>
+      <c r="K756" s="3" t="inlineStr"/>
+      <c r="L756" s="4" t="inlineStr">
+        <is>
+          <t>T1D88570</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B757" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000355</t>
+        </is>
+      </c>
+      <c r="C757" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D757" s="4" t="inlineStr">
+        <is>
+          <t>AD Bhubaneshwar</t>
+        </is>
+      </c>
+      <c r="E757" s="4" t="inlineStr">
+        <is>
+          <t>Rakesh Nigam</t>
+        </is>
+      </c>
+      <c r="F757" s="4" t="inlineStr">
+        <is>
+          <t>ADITYA MOTORS</t>
+        </is>
+      </c>
+      <c r="G757" s="4" t="inlineStr">
+        <is>
+          <t>CUTTACK</t>
+        </is>
+      </c>
+      <c r="H757" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I757" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J757" s="4" t="inlineStr"/>
+      <c r="K757" s="3" t="inlineStr"/>
+      <c r="L757" s="4" t="inlineStr">
+        <is>
+          <t>T2C48500</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B758" s="4" t="inlineStr">
+        <is>
+          <t>LYL27A000054</t>
+        </is>
+      </c>
+      <c r="C758" s="4" t="inlineStr">
+        <is>
+          <t>25 Jun 2026</t>
+        </is>
+      </c>
+      <c r="D758" s="4" t="inlineStr">
+        <is>
+          <t>AD Raipur</t>
+        </is>
+      </c>
+      <c r="E758" s="4" t="inlineStr">
+        <is>
+          <t>Rohit Gajendra</t>
+        </is>
+      </c>
+      <c r="F758" s="4" t="inlineStr">
+        <is>
+          <t>RALAS AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="G758" s="4" t="inlineStr">
+        <is>
+          <t>DHAMTARI</t>
+        </is>
+      </c>
+      <c r="H758" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I758" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J758" s="4" t="inlineStr">
+        <is>
+          <t>Disclaimer Validation Failed: Disclaimer customer name 'Chandrashekhar Sahu' does not match claim customer 'Rohit Gajendra'; Disclaimer old vehicle registration number does not match portal registration 'UP16Q3936'; Disclaimer new vehicle chassis does not match claim chassis 'T2D72269' (Extracted: 'New Vehicle Model: MAHINDRA BOLERO B6 BS-VI | Chassis Number: T6D23737 | Engine Number: TVT6D49262'); Disclaimer new vehicle model does not match portal model group 'XUV3XO' (Extracted: 'New Vehicle Model: MAHINDRA BOLERO B6 BS-VI | Chassis Number: T6D23737 | Engine Number: TVT6D49262')
+Invoice Validation Failed: Invoice customer name 'CHANDRASHEKHAR SAHU' does not match claim customer 'Rohit Gajendra'
+OEM Document Validation Failed: New Chassis mismatch (Document Chassis: 'MA1XL2TVXT6D23737' does not match last 8 digits of dashboard: 'T2D72269')
+COD Document Validation Failed: COD Certificate No 'COD20260520HR43B6163' does not match expected old chassis 'COD20260520UP16Q3936'; Portal customer name 'Rohit Gajendra' not found from top to bottom in COD document (Extracted: 'CHANDRASHEKHAR SAHU'); COD Registration No 'HR43B6163' does not match expected old vehicle registration 'UP16Q3936'</t>
+        </is>
+      </c>
+      <c r="K758" s="3" t="inlineStr"/>
+      <c r="L758" s="4" t="inlineStr">
+        <is>
+          <t>T2D72269</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
zone wise north and east
</commit_message>
<xml_diff>
--- a/kyc_process_results.xlsx
+++ b/kyc_process_results.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L796"/>
+  <dimension ref="A1:L800"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46573,6 +46573,228 @@
         </is>
       </c>
     </row>
+    <row r="797">
+      <c r="A797" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B797" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000069</t>
+        </is>
+      </c>
+      <c r="C797" s="4" t="inlineStr">
+        <is>
+          <t>08 Jul 2026</t>
+        </is>
+      </c>
+      <c r="D797" s="4" t="inlineStr">
+        <is>
+          <t>AD Guwahati</t>
+        </is>
+      </c>
+      <c r="E797" s="4" t="inlineStr">
+        <is>
+          <t>Ajit Majumdar</t>
+        </is>
+      </c>
+      <c r="F797" s="4" t="inlineStr">
+        <is>
+          <t>PODDAR AUTOCORP PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="G797" s="4" t="inlineStr">
+        <is>
+          <t>GUWAHATI 3S</t>
+        </is>
+      </c>
+      <c r="H797" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I797" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J797" s="4" t="inlineStr">
+        <is>
+          <t>OEM Document Validation Failed: Certificate No mismatch (Document Certificate No: 'COD20250034S01AD1927' does not match old vehicle registration: 'AS01AD1927')</t>
+        </is>
+      </c>
+      <c r="K797" s="3" t="inlineStr"/>
+      <c r="L797" s="4" t="inlineStr">
+        <is>
+          <t>T2E91998</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B798" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000069</t>
+        </is>
+      </c>
+      <c r="C798" s="4" t="inlineStr">
+        <is>
+          <t>08 Jul 2026</t>
+        </is>
+      </c>
+      <c r="D798" s="4" t="inlineStr">
+        <is>
+          <t>AD Guwahati</t>
+        </is>
+      </c>
+      <c r="E798" s="4" t="inlineStr">
+        <is>
+          <t>Ajit Majumdar</t>
+        </is>
+      </c>
+      <c r="F798" s="4" t="inlineStr">
+        <is>
+          <t>PODDAR AUTOCORP PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="G798" s="4" t="inlineStr">
+        <is>
+          <t>GUWAHATI 3S</t>
+        </is>
+      </c>
+      <c r="H798" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I798" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J798" s="4" t="inlineStr">
+        <is>
+          <t>OEM Document Validation Failed: Certificate No mismatch (Document Certificate No: 'AS01GU7475' does not match old vehicle registration: 'AS01AD1927')</t>
+        </is>
+      </c>
+      <c r="K798" s="3" t="inlineStr"/>
+      <c r="L798" s="4" t="inlineStr">
+        <is>
+          <t>T2E91998</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B799" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000069</t>
+        </is>
+      </c>
+      <c r="C799" s="4" t="inlineStr">
+        <is>
+          <t>08 Jul 2026</t>
+        </is>
+      </c>
+      <c r="D799" s="4" t="inlineStr">
+        <is>
+          <t>AD Guwahati</t>
+        </is>
+      </c>
+      <c r="E799" s="4" t="inlineStr">
+        <is>
+          <t>Ajit Majumdar</t>
+        </is>
+      </c>
+      <c r="F799" s="4" t="inlineStr">
+        <is>
+          <t>PODDAR AUTOCORP PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="G799" s="4" t="inlineStr">
+        <is>
+          <t>GUWAHATI 3S</t>
+        </is>
+      </c>
+      <c r="H799" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I799" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J799" s="4" t="inlineStr"/>
+      <c r="K799" s="3" t="inlineStr"/>
+      <c r="L799" s="4" t="inlineStr">
+        <is>
+          <t>T2E91998</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B800" s="4" t="inlineStr">
+        <is>
+          <t>LYL27B000069</t>
+        </is>
+      </c>
+      <c r="C800" s="4" t="inlineStr">
+        <is>
+          <t>08 Jul 2026</t>
+        </is>
+      </c>
+      <c r="D800" s="4" t="inlineStr">
+        <is>
+          <t>AD Guwahati</t>
+        </is>
+      </c>
+      <c r="E800" s="4" t="inlineStr">
+        <is>
+          <t>Ajit Majumdar</t>
+        </is>
+      </c>
+      <c r="F800" s="4" t="inlineStr">
+        <is>
+          <t>PODDAR AUTOCORP PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="G800" s="4" t="inlineStr">
+        <is>
+          <t>GUWAHATI 3S</t>
+        </is>
+      </c>
+      <c r="H800" s="4" t="inlineStr">
+        <is>
+          <t>Scrappage Bonus</t>
+        </is>
+      </c>
+      <c r="I800" s="9" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="J800" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Validation Failed: LLM Extraction Failed
+Ledger Validation Failed: LLM Extraction Failed
+OEM Document Validation Failed: OpenAI Error: 400 Client Error: Bad Request for url: https://api.anthropic.com/v1/messages</t>
+        </is>
+      </c>
+      <c r="K800" s="3" t="inlineStr"/>
+      <c r="L800" s="4" t="inlineStr">
+        <is>
+          <t>T2E91998</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>